<commit_message>
Actualizacion de campos en las matrices correccion
</commit_message>
<xml_diff>
--- a/static/excel_files/IOS_IOSMX.xlsx
+++ b/static/excel_files/IOS_IOSMX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesusalberca/Desktop/qc_matrix_generator/static/excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4FA1D6-CCD2-CF44-8715-1641781ED9C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E0B1F1-E81A-8F4D-A46E-3510D3943A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20620" yWindow="660" windowWidth="30420" windowHeight="20780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1302,6 +1302,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" ht="15">
+      <c r="A2" s="5"/>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1320,11 +1321,12 @@
       <c r="I2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="4"/>
+      <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="3"/>
     </row>
     <row r="3" spans="1:12" ht="15">
+      <c r="A3" s="5"/>
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
@@ -1343,11 +1345,12 @@
       <c r="I3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="4"/>
+      <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
     </row>
     <row r="4" spans="1:12" ht="15">
+      <c r="A4" s="3"/>
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
@@ -1366,11 +1369,12 @@
       <c r="I4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="4"/>
+      <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
     </row>
     <row r="5" spans="1:12" ht="15">
+      <c r="A5" s="5"/>
       <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
@@ -1389,11 +1393,12 @@
       <c r="I5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="4"/>
+      <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="3"/>
     </row>
     <row r="6" spans="1:12" ht="15">
+      <c r="A6" s="5"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1412,11 +1417,12 @@
       <c r="I6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J6" s="4"/>
+      <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="15">
+      <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
@@ -1435,11 +1441,12 @@
       <c r="I7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J7" s="4"/>
+      <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
     </row>
     <row r="8" spans="1:12" ht="15">
+      <c r="A8" s="5"/>
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1458,11 +1465,12 @@
       <c r="I8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="4"/>
+      <c r="J8" s="5"/>
       <c r="K8" s="5"/>
       <c r="L8" s="3"/>
     </row>
     <row r="9" spans="1:12" ht="15">
+      <c r="A9" s="3"/>
       <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
@@ -1481,11 +1489,12 @@
       <c r="I9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J9" s="4"/>
+      <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="15">
+      <c r="A10" s="5"/>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1504,11 +1513,12 @@
       <c r="I10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="4"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="3"/>
     </row>
     <row r="11" spans="1:12" ht="15">
+      <c r="A11" s="3"/>
       <c r="B11" s="6" t="s">
         <v>3</v>
       </c>
@@ -1527,11 +1537,12 @@
       <c r="I11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J11" s="4"/>
+      <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
     </row>
     <row r="12" spans="1:12" ht="15">
+      <c r="A12" s="5"/>
       <c r="B12" s="1" t="s">
         <v>3</v>
       </c>
@@ -1550,11 +1561,12 @@
       <c r="I12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J12" s="4"/>
+      <c r="J12" s="5"/>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="15">
+      <c r="A13" s="3"/>
       <c r="B13" s="6" t="s">
         <v>9</v>
       </c>
@@ -1573,11 +1585,12 @@
       <c r="I13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J13" s="4"/>
+      <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
     </row>
     <row r="14" spans="1:12" ht="15">
+      <c r="A14" s="5"/>
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
@@ -1596,11 +1609,12 @@
       <c r="I14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J14" s="4"/>
+      <c r="J14" s="5"/>
       <c r="K14" s="5"/>
       <c r="L14" s="3"/>
     </row>
     <row r="15" spans="1:12" ht="15">
+      <c r="A15" s="5"/>
       <c r="B15" s="6" t="s">
         <v>9</v>
       </c>
@@ -1619,11 +1633,12 @@
       <c r="I15" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J15" s="4"/>
+      <c r="J15" s="5"/>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="15">
+      <c r="A16" s="5"/>
       <c r="B16" s="1" t="s">
         <v>9</v>
       </c>
@@ -1642,11 +1657,12 @@
       <c r="I16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J16" s="4"/>
+      <c r="J16" s="5"/>
       <c r="K16" s="5"/>
       <c r="L16" s="3"/>
     </row>
-    <row r="17" spans="2:12" ht="15">
+    <row r="17" spans="1:12" ht="15">
+      <c r="A17" s="5"/>
       <c r="B17" s="6" t="s">
         <v>3</v>
       </c>
@@ -1665,11 +1681,12 @@
       <c r="I17" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J17" s="4"/>
+      <c r="J17" s="5"/>
       <c r="K17" s="5"/>
       <c r="L17" s="3"/>
     </row>
-    <row r="18" spans="2:12" ht="15">
+    <row r="18" spans="1:12" ht="15">
+      <c r="A18" s="5"/>
       <c r="B18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1688,11 +1705,12 @@
       <c r="I18" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J18" s="4"/>
+      <c r="J18" s="5"/>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
     </row>
-    <row r="19" spans="2:12" ht="15">
+    <row r="19" spans="1:12" ht="15">
+      <c r="A19" s="3"/>
       <c r="B19" s="6" t="s">
         <v>9</v>
       </c>
@@ -1711,11 +1729,12 @@
       <c r="I19" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J19" s="4"/>
+      <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
     </row>
-    <row r="20" spans="2:12" ht="15">
+    <row r="20" spans="1:12" ht="15">
+      <c r="A20" s="5"/>
       <c r="B20" s="1" t="s">
         <v>3</v>
       </c>
@@ -1734,11 +1753,12 @@
       <c r="I20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J20" s="4"/>
+      <c r="J20" s="5"/>
       <c r="K20" s="5"/>
       <c r="L20" s="3"/>
     </row>
-    <row r="21" spans="2:12" ht="15">
+    <row r="21" spans="1:12" ht="15">
+      <c r="A21" s="5"/>
       <c r="B21" s="6" t="s">
         <v>3</v>
       </c>
@@ -1757,11 +1777,12 @@
       <c r="I21" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J21" s="4"/>
+      <c r="J21" s="5"/>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
     </row>
-    <row r="22" spans="2:12" ht="30">
+    <row r="22" spans="1:12" ht="30">
+      <c r="A22" s="5"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -1780,11 +1801,12 @@
       <c r="I22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J22" s="4"/>
+      <c r="J22" s="5"/>
       <c r="K22" s="5"/>
       <c r="L22" s="3"/>
     </row>
-    <row r="23" spans="2:12" ht="15">
+    <row r="23" spans="1:12" ht="15">
+      <c r="A23" s="5"/>
       <c r="B23" s="6" t="s">
         <v>9</v>
       </c>
@@ -1803,11 +1825,12 @@
       <c r="I23" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J23" s="4"/>
+      <c r="J23" s="5"/>
       <c r="K23" s="5"/>
       <c r="L23" s="3"/>
     </row>
-    <row r="24" spans="2:12" ht="30">
+    <row r="24" spans="1:12" ht="30">
+      <c r="A24" s="5"/>
       <c r="B24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1826,11 +1849,12 @@
       <c r="I24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J24" s="4"/>
+      <c r="J24" s="5"/>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
     </row>
-    <row r="25" spans="2:12" ht="15">
+    <row r="25" spans="1:12" ht="15">
+      <c r="A25" s="5"/>
       <c r="B25" s="6" t="s">
         <v>9</v>
       </c>
@@ -1849,11 +1873,12 @@
       <c r="I25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J25" s="4"/>
+      <c r="J25" s="5"/>
       <c r="K25" s="5"/>
       <c r="L25" s="3"/>
     </row>
-    <row r="26" spans="2:12" ht="15">
+    <row r="26" spans="1:12" ht="15">
+      <c r="A26" s="3"/>
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
@@ -1872,11 +1897,12 @@
       <c r="I26" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J26" s="4"/>
+      <c r="J26" s="3"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
     </row>
-    <row r="27" spans="2:12" ht="15">
+    <row r="27" spans="1:12" ht="15">
+      <c r="A27" s="3"/>
       <c r="B27" s="6" t="s">
         <v>9</v>
       </c>
@@ -1895,11 +1921,12 @@
       <c r="I27" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J27" s="4"/>
+      <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="5"/>
     </row>
-    <row r="28" spans="2:12" ht="15">
+    <row r="28" spans="1:12" ht="15">
+      <c r="A28" s="5"/>
       <c r="B28" s="1" t="s">
         <v>9</v>
       </c>
@@ -1918,11 +1945,12 @@
       <c r="I28" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J28" s="4"/>
+      <c r="J28" s="5"/>
       <c r="K28" s="5"/>
       <c r="L28" s="3"/>
     </row>
-    <row r="29" spans="2:12" ht="15">
+    <row r="29" spans="1:12" ht="15">
+      <c r="A29" s="5"/>
       <c r="B29" s="6" t="s">
         <v>39</v>
       </c>
@@ -1941,11 +1969,12 @@
       <c r="I29" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J29" s="4"/>
+      <c r="J29" s="5"/>
       <c r="K29" s="5"/>
       <c r="L29" s="3"/>
     </row>
-    <row r="30" spans="2:12" ht="15">
+    <row r="30" spans="1:12" ht="15">
+      <c r="A30" s="5"/>
       <c r="B30" s="1" t="s">
         <v>39</v>
       </c>
@@ -1964,11 +1993,12 @@
       <c r="I30" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J30" s="4"/>
+      <c r="J30" s="5"/>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
     </row>
-    <row r="31" spans="2:12" ht="15">
+    <row r="31" spans="1:12" ht="15">
+      <c r="A31" s="5"/>
       <c r="B31" s="6" t="s">
         <v>39</v>
       </c>
@@ -1987,11 +2017,12 @@
       <c r="I31" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J31" s="4"/>
+      <c r="J31" s="5"/>
       <c r="K31" s="5"/>
       <c r="L31" s="3"/>
     </row>
-    <row r="32" spans="2:12" ht="15">
+    <row r="32" spans="1:12" ht="15">
+      <c r="A32" s="5"/>
       <c r="B32" s="1" t="s">
         <v>39</v>
       </c>
@@ -2010,11 +2041,12 @@
       <c r="I32" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J32" s="4"/>
+      <c r="J32" s="5"/>
       <c r="K32" s="5"/>
       <c r="L32" s="3"/>
     </row>
-    <row r="33" spans="2:12" ht="15">
+    <row r="33" spans="1:12" ht="15">
+      <c r="A33" s="5"/>
       <c r="B33" s="6" t="s">
         <v>39</v>
       </c>
@@ -2033,11 +2065,12 @@
       <c r="I33" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J33" s="4"/>
+      <c r="J33" s="5"/>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
     </row>
-    <row r="34" spans="2:12" ht="15">
+    <row r="34" spans="1:12" ht="15">
+      <c r="A34" s="5"/>
       <c r="B34" s="1" t="s">
         <v>39</v>
       </c>
@@ -2056,11 +2089,12 @@
       <c r="I34" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J34" s="4"/>
+      <c r="J34" s="5"/>
       <c r="K34" s="5"/>
       <c r="L34" s="3"/>
     </row>
-    <row r="35" spans="2:12" ht="30">
+    <row r="35" spans="1:12" ht="30">
+      <c r="A35" s="5"/>
       <c r="B35" s="6" t="s">
         <v>39</v>
       </c>
@@ -2079,11 +2113,12 @@
       <c r="I35" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J35" s="4"/>
+      <c r="J35" s="5"/>
       <c r="K35" s="5"/>
       <c r="L35" s="3"/>
     </row>
-    <row r="36" spans="2:12" ht="15">
+    <row r="36" spans="1:12" ht="15">
+      <c r="A36" s="5"/>
       <c r="B36" s="1" t="s">
         <v>39</v>
       </c>
@@ -2102,11 +2137,12 @@
       <c r="I36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J36" s="4"/>
+      <c r="J36" s="5"/>
       <c r="K36" s="5"/>
       <c r="L36" s="5"/>
     </row>
-    <row r="37" spans="2:12" ht="30">
+    <row r="37" spans="1:12" ht="30">
+      <c r="A37" s="5"/>
       <c r="B37" s="6" t="s">
         <v>9</v>
       </c>
@@ -2125,11 +2161,12 @@
       <c r="I37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J37" s="4"/>
+      <c r="J37" s="5"/>
       <c r="K37" s="5"/>
       <c r="L37" s="3"/>
     </row>
-    <row r="38" spans="2:12" ht="15">
+    <row r="38" spans="1:12" ht="15">
+      <c r="A38" s="5"/>
       <c r="B38" s="1" t="s">
         <v>9</v>
       </c>
@@ -2148,11 +2185,12 @@
       <c r="I38" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J38" s="4"/>
+      <c r="J38" s="5"/>
       <c r="K38" s="5"/>
       <c r="L38" s="3"/>
     </row>
-    <row r="39" spans="2:12" ht="30">
+    <row r="39" spans="1:12" ht="30">
+      <c r="A39" s="5"/>
       <c r="B39" s="6" t="s">
         <v>9</v>
       </c>
@@ -2171,11 +2209,12 @@
       <c r="I39" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J39" s="4"/>
+      <c r="J39" s="5"/>
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
     </row>
-    <row r="40" spans="2:12" ht="15">
+    <row r="40" spans="1:12" ht="15">
+      <c r="A40" s="5"/>
       <c r="B40" s="1" t="s">
         <v>39</v>
       </c>
@@ -2194,11 +2233,12 @@
       <c r="I40" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J40" s="4"/>
+      <c r="J40" s="5"/>
       <c r="K40" s="5"/>
       <c r="L40" s="3"/>
     </row>
-    <row r="41" spans="2:12" ht="30">
+    <row r="41" spans="1:12" ht="30">
+      <c r="A41" s="5"/>
       <c r="B41" s="6" t="s">
         <v>9</v>
       </c>
@@ -2217,11 +2257,12 @@
       <c r="I41" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J41" s="4"/>
+      <c r="J41" s="5"/>
       <c r="K41" s="5"/>
       <c r="L41" s="3"/>
     </row>
-    <row r="42" spans="2:12" ht="15">
+    <row r="42" spans="1:12" ht="15">
+      <c r="A42" s="5"/>
       <c r="B42" s="1" t="s">
         <v>39</v>
       </c>
@@ -2240,11 +2281,12 @@
       <c r="I42" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J42" s="4"/>
+      <c r="J42" s="5"/>
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
     </row>
-    <row r="43" spans="2:12" ht="15">
+    <row r="43" spans="1:12" ht="15">
+      <c r="A43" s="3"/>
       <c r="B43" s="6" t="s">
         <v>39</v>
       </c>
@@ -2263,11 +2305,12 @@
       <c r="I43" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J43" s="4"/>
+      <c r="J43" s="3"/>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
     </row>
-    <row r="44" spans="2:12" ht="30">
+    <row r="44" spans="1:12" ht="30">
+      <c r="A44" s="3"/>
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
@@ -2286,11 +2329,12 @@
       <c r="I44" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J44" s="4"/>
+      <c r="J44" s="3"/>
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
     </row>
-    <row r="45" spans="2:12" ht="15">
+    <row r="45" spans="1:12" ht="15">
+      <c r="A45" s="3"/>
       <c r="B45" s="6" t="s">
         <v>9</v>
       </c>
@@ -2309,11 +2353,12 @@
       <c r="I45" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J45" s="4"/>
+      <c r="J45" s="3"/>
       <c r="K45" s="3"/>
       <c r="L45" s="5"/>
     </row>
-    <row r="46" spans="2:12" ht="15">
+    <row r="46" spans="1:12" ht="15">
+      <c r="A46" s="3"/>
       <c r="B46" s="1" t="s">
         <v>39</v>
       </c>
@@ -2332,11 +2377,12 @@
       <c r="I46" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J46" s="4"/>
+      <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
     </row>
-    <row r="47" spans="2:12" ht="15">
+    <row r="47" spans="1:12" ht="15">
+      <c r="A47" s="3"/>
       <c r="B47" s="6" t="s">
         <v>39</v>
       </c>
@@ -2355,11 +2401,12 @@
       <c r="I47" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J47" s="4"/>
+      <c r="J47" s="3"/>
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
     </row>
-    <row r="48" spans="2:12" ht="15">
+    <row r="48" spans="1:12" ht="15">
+      <c r="A48" s="5"/>
       <c r="B48" s="1" t="s">
         <v>39</v>
       </c>
@@ -2378,11 +2425,12 @@
       <c r="I48" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J48" s="4"/>
+      <c r="J48" s="5"/>
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
     </row>
-    <row r="49" spans="2:12" ht="15">
+    <row r="49" spans="1:12" ht="15">
+      <c r="A49" s="3"/>
       <c r="B49" s="6" t="s">
         <v>39</v>
       </c>
@@ -2401,11 +2449,12 @@
       <c r="I49" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J49" s="4"/>
+      <c r="J49" s="3"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
     </row>
-    <row r="50" spans="2:12" ht="30">
+    <row r="50" spans="1:12" ht="30">
+      <c r="A50" s="5"/>
       <c r="B50" s="1" t="s">
         <v>39</v>
       </c>
@@ -2424,11 +2473,12 @@
       <c r="I50" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J50" s="4"/>
+      <c r="J50" s="5"/>
       <c r="K50" s="5"/>
       <c r="L50" s="3"/>
     </row>
-    <row r="51" spans="2:12" ht="15">
+    <row r="51" spans="1:12" ht="15">
+      <c r="A51" s="5"/>
       <c r="B51" s="6" t="s">
         <v>39</v>
       </c>
@@ -2447,11 +2497,12 @@
       <c r="I51" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J51" s="4"/>
+      <c r="J51" s="5"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5"/>
     </row>
-    <row r="52" spans="2:12" ht="30">
+    <row r="52" spans="1:12" ht="30">
+      <c r="A52" s="5"/>
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
@@ -2470,11 +2521,12 @@
       <c r="I52" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J52" s="4"/>
+      <c r="J52" s="5"/>
       <c r="K52" s="5"/>
       <c r="L52" s="3"/>
     </row>
-    <row r="53" spans="2:12" ht="30">
+    <row r="53" spans="1:12" ht="30">
+      <c r="A53" s="5"/>
       <c r="B53" s="6" t="s">
         <v>9</v>
       </c>
@@ -2493,11 +2545,12 @@
       <c r="I53" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J53" s="4"/>
+      <c r="J53" s="5"/>
       <c r="K53" s="5"/>
       <c r="L53" s="3"/>
     </row>
-    <row r="54" spans="2:12" ht="15">
+    <row r="54" spans="1:12" ht="15">
+      <c r="A54" s="5"/>
       <c r="B54" s="1" t="s">
         <v>9</v>
       </c>
@@ -2516,11 +2569,12 @@
       <c r="I54" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J54" s="4"/>
+      <c r="J54" s="5"/>
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
     </row>
-    <row r="55" spans="2:12" ht="15">
+    <row r="55" spans="1:12" ht="15">
+      <c r="A55" s="5"/>
       <c r="B55" s="6" t="s">
         <v>39</v>
       </c>
@@ -2539,11 +2593,12 @@
       <c r="I55" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J55" s="4"/>
+      <c r="J55" s="5"/>
       <c r="K55" s="5"/>
       <c r="L55" s="3"/>
     </row>
-    <row r="56" spans="2:12" ht="15">
+    <row r="56" spans="1:12" ht="15">
+      <c r="A56" s="5"/>
       <c r="B56" s="1" t="s">
         <v>39</v>
       </c>
@@ -2562,11 +2617,12 @@
       <c r="I56" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J56" s="4"/>
+      <c r="J56" s="5"/>
       <c r="K56" s="5"/>
       <c r="L56" s="3"/>
     </row>
-    <row r="57" spans="2:12" ht="15">
+    <row r="57" spans="1:12" ht="15">
+      <c r="A57" s="5"/>
       <c r="B57" s="6" t="s">
         <v>39</v>
       </c>
@@ -2585,11 +2641,12 @@
       <c r="I57" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J57" s="4"/>
+      <c r="J57" s="5"/>
       <c r="K57" s="5"/>
       <c r="L57" s="5"/>
     </row>
-    <row r="58" spans="2:12" ht="15">
+    <row r="58" spans="1:12" ht="15">
+      <c r="A58" s="5"/>
       <c r="B58" s="1" t="s">
         <v>39</v>
       </c>
@@ -2608,11 +2665,12 @@
       <c r="I58" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J58" s="4"/>
+      <c r="J58" s="5"/>
       <c r="K58" s="5"/>
       <c r="L58" s="3"/>
     </row>
-    <row r="59" spans="2:12" ht="30">
+    <row r="59" spans="1:12" ht="30">
+      <c r="A59" s="5"/>
       <c r="B59" s="6" t="s">
         <v>39</v>
       </c>
@@ -2631,11 +2689,12 @@
       <c r="I59" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J59" s="4"/>
+      <c r="J59" s="5"/>
       <c r="K59" s="5"/>
       <c r="L59" s="3"/>
     </row>
-    <row r="60" spans="2:12" ht="15">
+    <row r="60" spans="1:12" ht="15">
+      <c r="A60" s="5"/>
       <c r="B60" s="1" t="s">
         <v>39</v>
       </c>
@@ -2654,11 +2713,12 @@
       <c r="I60" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J60" s="4"/>
+      <c r="J60" s="5"/>
       <c r="K60" s="5"/>
       <c r="L60" s="5"/>
     </row>
-    <row r="61" spans="2:12" ht="15">
+    <row r="61" spans="1:12" ht="15">
+      <c r="A61" s="5"/>
       <c r="B61" s="6" t="s">
         <v>39</v>
       </c>
@@ -2677,11 +2737,12 @@
       <c r="I61" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J61" s="4"/>
+      <c r="J61" s="5"/>
       <c r="K61" s="5"/>
       <c r="L61" s="3"/>
     </row>
-    <row r="62" spans="2:12" ht="15">
+    <row r="62" spans="1:12" ht="15">
+      <c r="A62" s="5"/>
       <c r="B62" s="1" t="s">
         <v>39</v>
       </c>
@@ -2700,11 +2761,12 @@
       <c r="I62" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J62" s="4"/>
+      <c r="J62" s="5"/>
       <c r="K62" s="5"/>
       <c r="L62" s="3"/>
     </row>
-    <row r="63" spans="2:12" ht="30">
+    <row r="63" spans="1:12" ht="30">
+      <c r="A63" s="5"/>
       <c r="B63" s="6" t="s">
         <v>9</v>
       </c>
@@ -2723,11 +2785,12 @@
       <c r="I63" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J63" s="4"/>
+      <c r="J63" s="5"/>
       <c r="K63" s="5"/>
       <c r="L63" s="5"/>
     </row>
-    <row r="64" spans="2:12" ht="30">
+    <row r="64" spans="1:12" ht="30">
+      <c r="A64" s="5"/>
       <c r="B64" s="1" t="s">
         <v>9</v>
       </c>
@@ -2746,11 +2809,12 @@
       <c r="I64" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J64" s="4"/>
+      <c r="J64" s="5"/>
       <c r="K64" s="5"/>
       <c r="L64" s="3"/>
     </row>
-    <row r="65" spans="2:12" ht="15">
+    <row r="65" spans="1:12" ht="15">
+      <c r="A65" s="5"/>
       <c r="B65" s="6" t="s">
         <v>9</v>
       </c>
@@ -2769,11 +2833,12 @@
       <c r="I65" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J65" s="4"/>
+      <c r="J65" s="5"/>
       <c r="K65" s="5"/>
       <c r="L65" s="3"/>
     </row>
-    <row r="66" spans="2:12" ht="45">
+    <row r="66" spans="1:12" ht="45">
+      <c r="A66" s="5"/>
       <c r="B66" s="1" t="s">
         <v>9</v>
       </c>
@@ -2792,11 +2857,12 @@
       <c r="I66" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J66" s="4"/>
+      <c r="J66" s="5"/>
       <c r="K66" s="5"/>
       <c r="L66" s="5"/>
     </row>
-    <row r="67" spans="2:12" ht="15">
+    <row r="67" spans="1:12" ht="15">
+      <c r="A67" s="5"/>
       <c r="B67" s="6" t="s">
         <v>9</v>
       </c>
@@ -2815,11 +2881,12 @@
       <c r="I67" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J67" s="4"/>
+      <c r="J67" s="5"/>
       <c r="K67" s="5"/>
       <c r="L67" s="3"/>
     </row>
-    <row r="68" spans="2:12" ht="30">
+    <row r="68" spans="1:12" ht="30">
+      <c r="A68" s="5"/>
       <c r="B68" s="1" t="s">
         <v>39</v>
       </c>
@@ -2838,11 +2905,12 @@
       <c r="I68" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J68" s="4"/>
+      <c r="J68" s="5"/>
       <c r="K68" s="5"/>
       <c r="L68" s="3"/>
     </row>
-    <row r="69" spans="2:12" ht="15">
+    <row r="69" spans="1:12" ht="15">
+      <c r="A69" s="5"/>
       <c r="B69" s="6" t="s">
         <v>39</v>
       </c>
@@ -2861,11 +2929,12 @@
       <c r="I69" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J69" s="4"/>
+      <c r="J69" s="5"/>
       <c r="K69" s="5"/>
       <c r="L69" s="5"/>
     </row>
-    <row r="70" spans="2:12" ht="30">
+    <row r="70" spans="1:12" ht="30">
+      <c r="A70" s="5"/>
       <c r="B70" s="1" t="s">
         <v>9</v>
       </c>
@@ -2884,11 +2953,12 @@
       <c r="I70" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J70" s="4"/>
+      <c r="J70" s="5"/>
       <c r="K70" s="5"/>
       <c r="L70" s="3"/>
     </row>
-    <row r="71" spans="2:12" ht="15">
+    <row r="71" spans="1:12" ht="15">
+      <c r="A71" s="5"/>
       <c r="B71" s="6" t="s">
         <v>9</v>
       </c>
@@ -2907,11 +2977,12 @@
       <c r="I71" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J71" s="4"/>
+      <c r="J71" s="5"/>
       <c r="K71" s="5"/>
       <c r="L71" s="3"/>
     </row>
-    <row r="72" spans="2:12" ht="15">
+    <row r="72" spans="1:12" ht="15">
+      <c r="A72" s="5"/>
       <c r="B72" s="1" t="s">
         <v>9</v>
       </c>
@@ -2930,11 +3001,12 @@
       <c r="I72" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J72" s="4"/>
+      <c r="J72" s="5"/>
       <c r="K72" s="5"/>
       <c r="L72" s="5"/>
     </row>
-    <row r="73" spans="2:12" ht="30">
+    <row r="73" spans="1:12" ht="30">
+      <c r="A73" s="5"/>
       <c r="B73" s="6" t="s">
         <v>39</v>
       </c>
@@ -2953,11 +3025,12 @@
       <c r="I73" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J73" s="4"/>
+      <c r="J73" s="5"/>
       <c r="K73" s="5"/>
       <c r="L73" s="3"/>
     </row>
-    <row r="74" spans="2:12" ht="15">
+    <row r="74" spans="1:12" ht="15">
+      <c r="A74" s="5"/>
       <c r="B74" s="1" t="s">
         <v>39</v>
       </c>
@@ -2976,11 +3049,12 @@
       <c r="I74" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J74" s="4"/>
+      <c r="J74" s="5"/>
       <c r="K74" s="5"/>
       <c r="L74" s="3"/>
     </row>
-    <row r="75" spans="2:12" ht="30">
+    <row r="75" spans="1:12" ht="30">
+      <c r="A75" s="5"/>
       <c r="B75" s="6" t="s">
         <v>9</v>
       </c>
@@ -2999,11 +3073,12 @@
       <c r="I75" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J75" s="4"/>
+      <c r="J75" s="5"/>
       <c r="K75" s="5"/>
       <c r="L75" s="5"/>
     </row>
-    <row r="76" spans="2:12" ht="15">
+    <row r="76" spans="1:12" ht="15">
+      <c r="A76" s="5"/>
       <c r="B76" s="1" t="s">
         <v>9</v>
       </c>
@@ -3022,11 +3097,12 @@
       <c r="I76" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J76" s="4"/>
+      <c r="J76" s="5"/>
       <c r="K76" s="5"/>
       <c r="L76" s="3"/>
     </row>
-    <row r="77" spans="2:12" ht="15">
+    <row r="77" spans="1:12" ht="15">
+      <c r="A77" s="5"/>
       <c r="B77" s="6" t="s">
         <v>9</v>
       </c>
@@ -3045,11 +3121,12 @@
       <c r="I77" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J77" s="4"/>
+      <c r="J77" s="5"/>
       <c r="K77" s="5"/>
       <c r="L77" s="3"/>
     </row>
-    <row r="78" spans="2:12" ht="45">
+    <row r="78" spans="1:12" ht="45">
+      <c r="A78" s="5"/>
       <c r="B78" s="1" t="s">
         <v>9</v>
       </c>
@@ -3068,11 +3145,12 @@
       <c r="I78" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J78" s="4"/>
+      <c r="J78" s="5"/>
       <c r="K78" s="5"/>
       <c r="L78" s="5"/>
     </row>
-    <row r="79" spans="2:12" ht="15">
+    <row r="79" spans="1:12" ht="15">
+      <c r="A79" s="5"/>
       <c r="B79" s="6" t="s">
         <v>9</v>
       </c>
@@ -3091,11 +3169,12 @@
       <c r="I79" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J79" s="4"/>
+      <c r="J79" s="5"/>
       <c r="K79" s="5"/>
       <c r="L79" s="3"/>
     </row>
-    <row r="80" spans="2:12" ht="30">
+    <row r="80" spans="1:12" ht="30">
+      <c r="A80" s="5"/>
       <c r="B80" s="1" t="s">
         <v>39</v>
       </c>
@@ -3114,11 +3193,12 @@
       <c r="I80" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J80" s="4"/>
+      <c r="J80" s="5"/>
       <c r="K80" s="5"/>
       <c r="L80" s="3"/>
     </row>
-    <row r="81" spans="2:12" ht="15">
+    <row r="81" spans="1:12" ht="15">
+      <c r="A81" s="5"/>
       <c r="B81" s="6" t="s">
         <v>39</v>
       </c>
@@ -3137,11 +3217,12 @@
       <c r="I81" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J81" s="4"/>
+      <c r="J81" s="5"/>
       <c r="K81" s="5"/>
       <c r="L81" s="5"/>
     </row>
-    <row r="82" spans="2:12" ht="30">
+    <row r="82" spans="1:12" ht="30">
+      <c r="A82" s="5"/>
       <c r="B82" s="1" t="s">
         <v>9</v>
       </c>
@@ -3160,11 +3241,12 @@
       <c r="I82" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J82" s="4"/>
+      <c r="J82" s="5"/>
       <c r="K82" s="5"/>
       <c r="L82" s="3"/>
     </row>
-    <row r="83" spans="2:12" ht="15">
+    <row r="83" spans="1:12" ht="15">
+      <c r="A83" s="5"/>
       <c r="B83" s="6" t="s">
         <v>9</v>
       </c>
@@ -3183,11 +3265,12 @@
       <c r="I83" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J83" s="4"/>
+      <c r="J83" s="5"/>
       <c r="K83" s="5"/>
       <c r="L83" s="3"/>
     </row>
-    <row r="84" spans="2:12" ht="30">
+    <row r="84" spans="1:12" ht="30">
+      <c r="A84" s="5"/>
       <c r="B84" s="1" t="s">
         <v>9</v>
       </c>
@@ -3206,11 +3289,12 @@
       <c r="I84" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J84" s="4"/>
+      <c r="J84" s="5"/>
       <c r="K84" s="5"/>
       <c r="L84" s="5"/>
     </row>
-    <row r="85" spans="2:12" ht="30">
+    <row r="85" spans="1:12" ht="30">
+      <c r="A85" s="5"/>
       <c r="B85" s="6" t="s">
         <v>39</v>
       </c>
@@ -3229,11 +3313,12 @@
       <c r="I85" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J85" s="4"/>
+      <c r="J85" s="5"/>
       <c r="K85" s="5"/>
       <c r="L85" s="3"/>
     </row>
-    <row r="86" spans="2:12" ht="15">
+    <row r="86" spans="1:12" ht="15">
+      <c r="A86" s="5"/>
       <c r="B86" s="1" t="s">
         <v>39</v>
       </c>
@@ -3252,11 +3337,12 @@
       <c r="I86" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J86" s="4"/>
+      <c r="J86" s="5"/>
       <c r="K86" s="5"/>
       <c r="L86" s="3"/>
     </row>
-    <row r="87" spans="2:12" ht="30">
+    <row r="87" spans="1:12" ht="30">
+      <c r="A87" s="5"/>
       <c r="B87" s="6" t="s">
         <v>9</v>
       </c>
@@ -3275,11 +3361,12 @@
       <c r="I87" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J87" s="4"/>
+      <c r="J87" s="5"/>
       <c r="K87" s="5"/>
       <c r="L87" s="5"/>
     </row>
-    <row r="88" spans="2:12" ht="15">
+    <row r="88" spans="1:12" ht="15">
+      <c r="A88" s="5"/>
       <c r="B88" s="1" t="s">
         <v>9</v>
       </c>
@@ -3298,11 +3385,12 @@
       <c r="I88" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J88" s="4"/>
+      <c r="J88" s="5"/>
       <c r="K88" s="5"/>
       <c r="L88" s="3"/>
     </row>
-    <row r="89" spans="2:12" ht="45">
+    <row r="89" spans="1:12" ht="45">
+      <c r="A89" s="5"/>
       <c r="B89" s="6" t="s">
         <v>9</v>
       </c>
@@ -3321,11 +3409,12 @@
       <c r="I89" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J89" s="4"/>
+      <c r="J89" s="5"/>
       <c r="K89" s="5"/>
       <c r="L89" s="3"/>
     </row>
-    <row r="90" spans="2:12" ht="30">
+    <row r="90" spans="1:12" ht="30">
+      <c r="A90" s="5"/>
       <c r="B90" s="1" t="s">
         <v>39</v>
       </c>
@@ -3344,11 +3433,12 @@
       <c r="I90" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J90" s="4"/>
+      <c r="J90" s="5"/>
       <c r="K90" s="5"/>
       <c r="L90" s="5"/>
     </row>
-    <row r="91" spans="2:12" ht="15">
+    <row r="91" spans="1:12" ht="15">
+      <c r="A91" s="5"/>
       <c r="B91" s="6" t="s">
         <v>39</v>
       </c>
@@ -3367,11 +3457,12 @@
       <c r="I91" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J91" s="4"/>
+      <c r="J91" s="5"/>
       <c r="K91" s="5"/>
       <c r="L91" s="3"/>
     </row>
-    <row r="92" spans="2:12" ht="45">
+    <row r="92" spans="1:12" ht="45">
+      <c r="A92" s="5"/>
       <c r="B92" s="1" t="s">
         <v>9</v>
       </c>
@@ -3390,11 +3481,12 @@
       <c r="I92" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J92" s="4"/>
+      <c r="J92" s="5"/>
       <c r="K92" s="5"/>
       <c r="L92" s="3"/>
     </row>
-    <row r="93" spans="2:12" ht="15">
+    <row r="93" spans="1:12" ht="15">
+      <c r="A93" s="5"/>
       <c r="B93" s="6" t="s">
         <v>9</v>
       </c>
@@ -3413,11 +3505,12 @@
       <c r="I93" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J93" s="4"/>
+      <c r="J93" s="5"/>
       <c r="K93" s="5"/>
       <c r="L93" s="5"/>
     </row>
-    <row r="94" spans="2:12" ht="30">
+    <row r="94" spans="1:12" ht="30">
+      <c r="A94" s="5"/>
       <c r="B94" s="1" t="s">
         <v>39</v>
       </c>
@@ -3436,11 +3529,12 @@
       <c r="I94" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J94" s="4"/>
+      <c r="J94" s="5"/>
       <c r="K94" s="5"/>
       <c r="L94" s="3"/>
     </row>
-    <row r="95" spans="2:12" ht="15">
+    <row r="95" spans="1:12" ht="15">
+      <c r="A95" s="5"/>
       <c r="B95" s="6" t="s">
         <v>39</v>
       </c>
@@ -3459,11 +3553,12 @@
       <c r="I95" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J95" s="4"/>
+      <c r="J95" s="5"/>
       <c r="K95" s="5"/>
       <c r="L95" s="3"/>
     </row>
-    <row r="96" spans="2:12" ht="60">
+    <row r="96" spans="1:12" ht="60">
+      <c r="A96" s="5"/>
       <c r="B96" s="1" t="s">
         <v>9</v>
       </c>
@@ -3482,11 +3577,12 @@
       <c r="I96" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J96" s="4"/>
+      <c r="J96" s="5"/>
       <c r="K96" s="5"/>
       <c r="L96" s="5"/>
     </row>
-    <row r="97" spans="2:12" ht="30">
+    <row r="97" spans="1:12" ht="30">
+      <c r="A97" s="5"/>
       <c r="B97" s="6" t="s">
         <v>9</v>
       </c>
@@ -3505,11 +3601,12 @@
       <c r="I97" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J97" s="4"/>
+      <c r="J97" s="5"/>
       <c r="K97" s="5"/>
       <c r="L97" s="3"/>
     </row>
-    <row r="98" spans="2:12" ht="30">
+    <row r="98" spans="1:12" ht="30">
+      <c r="A98" s="5"/>
       <c r="B98" s="1" t="s">
         <v>39</v>
       </c>
@@ -3528,11 +3625,12 @@
       <c r="I98" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J98" s="4"/>
+      <c r="J98" s="5"/>
       <c r="K98" s="5"/>
       <c r="L98" s="3"/>
     </row>
-    <row r="99" spans="2:12" ht="30">
+    <row r="99" spans="1:12" ht="30">
+      <c r="A99" s="5"/>
       <c r="B99" s="6" t="s">
         <v>39</v>
       </c>
@@ -3551,11 +3649,12 @@
       <c r="I99" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J99" s="4"/>
+      <c r="J99" s="5"/>
       <c r="K99" s="5"/>
       <c r="L99" s="5"/>
     </row>
-    <row r="100" spans="2:12" ht="60">
+    <row r="100" spans="1:12" ht="60">
+      <c r="A100" s="5"/>
       <c r="B100" s="1" t="s">
         <v>9</v>
       </c>
@@ -3574,11 +3673,12 @@
       <c r="I100" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J100" s="4"/>
+      <c r="J100" s="5"/>
       <c r="K100" s="5"/>
       <c r="L100" s="3"/>
     </row>
-    <row r="101" spans="2:12" ht="30">
+    <row r="101" spans="1:12" ht="30">
+      <c r="A101" s="5"/>
       <c r="B101" s="6" t="s">
         <v>9</v>
       </c>
@@ -3597,11 +3697,12 @@
       <c r="I101" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J101" s="4"/>
+      <c r="J101" s="5"/>
       <c r="K101" s="5"/>
       <c r="L101" s="3"/>
     </row>
-    <row r="102" spans="2:12" ht="30">
+    <row r="102" spans="1:12" ht="30">
+      <c r="A102" s="5"/>
       <c r="B102" s="1" t="s">
         <v>39</v>
       </c>
@@ -3620,11 +3721,12 @@
       <c r="I102" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J102" s="4"/>
+      <c r="J102" s="5"/>
       <c r="K102" s="5"/>
       <c r="L102" s="5"/>
     </row>
-    <row r="103" spans="2:12" ht="15">
+    <row r="103" spans="1:12" ht="15">
+      <c r="A103" s="5"/>
       <c r="B103" s="6" t="s">
         <v>39</v>
       </c>
@@ -3643,11 +3745,12 @@
       <c r="I103" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J103" s="4"/>
+      <c r="J103" s="5"/>
       <c r="K103" s="5"/>
       <c r="L103" s="3"/>
     </row>
-    <row r="104" spans="2:12" ht="30">
+    <row r="104" spans="1:12" ht="30">
+      <c r="A104" s="5"/>
       <c r="B104" s="1" t="s">
         <v>3</v>
       </c>
@@ -3666,11 +3769,12 @@
       <c r="I104" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J104" s="4"/>
+      <c r="J104" s="5"/>
       <c r="K104" s="5"/>
       <c r="L104" s="3"/>
     </row>
-    <row r="105" spans="2:12" ht="30">
+    <row r="105" spans="1:12" ht="30">
+      <c r="A105" s="5"/>
       <c r="B105" s="6" t="s">
         <v>9</v>
       </c>
@@ -3689,11 +3793,12 @@
       <c r="I105" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J105" s="4"/>
+      <c r="J105" s="5"/>
       <c r="K105" s="5"/>
       <c r="L105" s="5"/>
     </row>
-    <row r="106" spans="2:12" ht="15">
+    <row r="106" spans="1:12" ht="15">
+      <c r="A106" s="5"/>
       <c r="B106" s="1" t="s">
         <v>9</v>
       </c>
@@ -3712,11 +3817,12 @@
       <c r="I106" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J106" s="4"/>
+      <c r="J106" s="5"/>
       <c r="K106" s="5"/>
       <c r="L106" s="3"/>
     </row>
-    <row r="107" spans="2:12" ht="45">
+    <row r="107" spans="1:12" ht="45">
+      <c r="A107" s="5"/>
       <c r="B107" s="6" t="s">
         <v>9</v>
       </c>
@@ -3735,11 +3841,12 @@
       <c r="I107" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J107" s="4"/>
+      <c r="J107" s="5"/>
       <c r="K107" s="5"/>
       <c r="L107" s="3"/>
     </row>
-    <row r="108" spans="2:12" ht="30">
+    <row r="108" spans="1:12" ht="30">
+      <c r="A108" s="5"/>
       <c r="B108" s="1" t="s">
         <v>9</v>
       </c>
@@ -3758,11 +3865,12 @@
       <c r="I108" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J108" s="4"/>
+      <c r="J108" s="5"/>
       <c r="K108" s="5"/>
       <c r="L108" s="5"/>
     </row>
-    <row r="109" spans="2:12" ht="30">
+    <row r="109" spans="1:12" ht="30">
+      <c r="A109" s="5"/>
       <c r="B109" s="6" t="s">
         <v>3</v>
       </c>
@@ -3781,11 +3889,12 @@
       <c r="I109" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J109" s="4"/>
+      <c r="J109" s="5"/>
       <c r="K109" s="5"/>
       <c r="L109" s="3"/>
     </row>
-    <row r="110" spans="2:12" ht="30">
+    <row r="110" spans="1:12" ht="30">
+      <c r="A110" s="5"/>
       <c r="B110" s="1" t="s">
         <v>3</v>
       </c>
@@ -3804,11 +3913,12 @@
       <c r="I110" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J110" s="4"/>
+      <c r="J110" s="5"/>
       <c r="K110" s="5"/>
       <c r="L110" s="3"/>
     </row>
-    <row r="111" spans="2:12" ht="30">
+    <row r="111" spans="1:12" ht="30">
+      <c r="A111" s="5"/>
       <c r="B111" s="6" t="s">
         <v>39</v>
       </c>
@@ -3827,11 +3937,12 @@
       <c r="I111" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J111" s="4"/>
+      <c r="J111" s="5"/>
       <c r="K111" s="5"/>
       <c r="L111" s="5"/>
     </row>
-    <row r="112" spans="2:12" ht="30">
+    <row r="112" spans="1:12" ht="30">
+      <c r="A112" s="5"/>
       <c r="B112" s="1" t="s">
         <v>3</v>
       </c>
@@ -3850,11 +3961,12 @@
       <c r="I112" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J112" s="4"/>
+      <c r="J112" s="5"/>
       <c r="K112" s="5"/>
       <c r="L112" s="3"/>
     </row>
-    <row r="113" spans="2:12" ht="15">
+    <row r="113" spans="1:12" ht="15">
+      <c r="A113" s="5"/>
       <c r="B113" s="6" t="s">
         <v>9</v>
       </c>
@@ -3873,11 +3985,12 @@
       <c r="I113" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J113" s="4"/>
+      <c r="J113" s="5"/>
       <c r="K113" s="5"/>
       <c r="L113" s="3"/>
     </row>
-    <row r="114" spans="2:12" ht="30">
+    <row r="114" spans="1:12" ht="30">
+      <c r="A114" s="5"/>
       <c r="B114" s="1" t="s">
         <v>3</v>
       </c>
@@ -3896,11 +4009,12 @@
       <c r="I114" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J114" s="4"/>
+      <c r="J114" s="5"/>
       <c r="K114" s="5"/>
       <c r="L114" s="5"/>
     </row>
-    <row r="115" spans="2:12" ht="30">
+    <row r="115" spans="1:12" ht="30">
+      <c r="A115" s="5"/>
       <c r="B115" s="6" t="s">
         <v>3</v>
       </c>
@@ -3919,11 +4033,12 @@
       <c r="I115" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J115" s="4"/>
+      <c r="J115" s="5"/>
       <c r="K115" s="5"/>
       <c r="L115" s="3"/>
     </row>
-    <row r="116" spans="2:12" ht="30">
+    <row r="116" spans="1:12" ht="30">
+      <c r="A116" s="5"/>
       <c r="B116" s="1" t="s">
         <v>3</v>
       </c>
@@ -3942,11 +4057,12 @@
       <c r="I116" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J116" s="4"/>
+      <c r="J116" s="5"/>
       <c r="K116" s="5"/>
       <c r="L116" s="3"/>
     </row>
-    <row r="117" spans="2:12" ht="15">
+    <row r="117" spans="1:12" ht="15">
+      <c r="A117" s="5"/>
       <c r="B117" s="6" t="s">
         <v>9</v>
       </c>
@@ -3965,11 +4081,12 @@
       <c r="I117" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J117" s="4"/>
+      <c r="J117" s="5"/>
       <c r="K117" s="5"/>
       <c r="L117" s="5"/>
     </row>
-    <row r="118" spans="2:12" ht="30">
+    <row r="118" spans="1:12" ht="30">
+      <c r="A118" s="5"/>
       <c r="B118" s="1" t="s">
         <v>3</v>
       </c>
@@ -3988,11 +4105,12 @@
       <c r="I118" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J118" s="4"/>
+      <c r="J118" s="5"/>
       <c r="K118" s="5"/>
       <c r="L118" s="3"/>
     </row>
-    <row r="119" spans="2:12" ht="30">
+    <row r="119" spans="1:12" ht="30">
+      <c r="A119" s="5"/>
       <c r="B119" s="6" t="s">
         <v>3</v>
       </c>
@@ -4011,11 +4129,12 @@
       <c r="I119" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J119" s="4"/>
+      <c r="J119" s="5"/>
       <c r="K119" s="5"/>
       <c r="L119" s="3"/>
     </row>
-    <row r="120" spans="2:12" ht="30">
+    <row r="120" spans="1:12" ht="30">
+      <c r="A120" s="5"/>
       <c r="B120" s="1" t="s">
         <v>3</v>
       </c>
@@ -4034,11 +4153,12 @@
       <c r="I120" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J120" s="4"/>
+      <c r="J120" s="5"/>
       <c r="K120" s="5"/>
       <c r="L120" s="5"/>
     </row>
-    <row r="121" spans="2:12" ht="30">
+    <row r="121" spans="1:12" ht="30">
+      <c r="A121" s="5"/>
       <c r="B121" s="6" t="s">
         <v>3</v>
       </c>
@@ -4057,11 +4177,12 @@
       <c r="I121" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J121" s="4"/>
+      <c r="J121" s="5"/>
       <c r="K121" s="5"/>
       <c r="L121" s="3"/>
     </row>
-    <row r="122" spans="2:12" ht="30">
+    <row r="122" spans="1:12" ht="30">
+      <c r="A122" s="5"/>
       <c r="B122" s="1" t="s">
         <v>3</v>
       </c>
@@ -4080,11 +4201,12 @@
       <c r="I122" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J122" s="4"/>
+      <c r="J122" s="5"/>
       <c r="K122" s="5"/>
       <c r="L122" s="3"/>
     </row>
-    <row r="123" spans="2:12" ht="15">
+    <row r="123" spans="1:12" ht="15">
+      <c r="A123" s="3"/>
       <c r="B123" s="6" t="s">
         <v>9</v>
       </c>
@@ -4103,11 +4225,12 @@
       <c r="I123" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J123" s="4"/>
+      <c r="J123" s="3"/>
       <c r="K123" s="3"/>
       <c r="L123" s="5"/>
     </row>
-    <row r="124" spans="2:12" ht="15">
+    <row r="124" spans="1:12" ht="15">
+      <c r="A124" s="5"/>
       <c r="B124" s="1" t="s">
         <v>9</v>
       </c>
@@ -4126,11 +4249,12 @@
       <c r="I124" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J124" s="4"/>
+      <c r="J124" s="5"/>
       <c r="K124" s="5"/>
       <c r="L124" s="3"/>
     </row>
-    <row r="125" spans="2:12" ht="30">
+    <row r="125" spans="1:12" ht="30">
+      <c r="A125" s="5"/>
       <c r="B125" s="6" t="s">
         <v>9</v>
       </c>
@@ -4149,11 +4273,12 @@
       <c r="I125" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J125" s="4"/>
+      <c r="J125" s="5"/>
       <c r="K125" s="5"/>
       <c r="L125" s="3"/>
     </row>
-    <row r="126" spans="2:12" ht="30">
+    <row r="126" spans="1:12" ht="30">
+      <c r="A126" s="5"/>
       <c r="B126" s="1" t="s">
         <v>9</v>
       </c>
@@ -4172,11 +4297,12 @@
       <c r="I126" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J126" s="4"/>
+      <c r="J126" s="5"/>
       <c r="K126" s="5"/>
       <c r="L126" s="5"/>
     </row>
-    <row r="127" spans="2:12" ht="15">
+    <row r="127" spans="1:12" ht="15">
+      <c r="A127" s="5"/>
       <c r="B127" s="6" t="s">
         <v>3</v>
       </c>
@@ -4195,11 +4321,12 @@
       <c r="I127" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J127" s="4"/>
+      <c r="J127" s="5"/>
       <c r="K127" s="5"/>
       <c r="L127" s="3"/>
     </row>
-    <row r="128" spans="2:12" ht="15">
+    <row r="128" spans="1:12" ht="15">
+      <c r="A128" s="5"/>
       <c r="B128" s="1" t="s">
         <v>3</v>
       </c>
@@ -4218,11 +4345,12 @@
       <c r="I128" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J128" s="4"/>
+      <c r="J128" s="5"/>
       <c r="K128" s="5"/>
       <c r="L128" s="3"/>
     </row>
-    <row r="129" spans="2:12" ht="15">
+    <row r="129" spans="1:12" ht="15">
+      <c r="A129" s="5"/>
       <c r="B129" s="6" t="s">
         <v>9</v>
       </c>
@@ -4241,11 +4369,12 @@
       <c r="I129" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J129" s="4"/>
+      <c r="J129" s="5"/>
       <c r="K129" s="5"/>
       <c r="L129" s="5"/>
     </row>
-    <row r="130" spans="2:12" ht="15">
+    <row r="130" spans="1:12" ht="15">
+      <c r="A130" s="5"/>
       <c r="B130" s="1" t="s">
         <v>3</v>
       </c>
@@ -4264,11 +4393,12 @@
       <c r="I130" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J130" s="4"/>
+      <c r="J130" s="5"/>
       <c r="K130" s="5"/>
       <c r="L130" s="3"/>
     </row>
-    <row r="131" spans="2:12" ht="15">
+    <row r="131" spans="1:12" ht="15">
+      <c r="A131" s="3"/>
       <c r="B131" s="6" t="s">
         <v>3</v>
       </c>
@@ -4287,11 +4417,12 @@
       <c r="I131" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J131" s="4"/>
+      <c r="J131" s="3"/>
       <c r="K131" s="3"/>
       <c r="L131" s="3"/>
     </row>
-    <row r="132" spans="2:12" ht="15">
+    <row r="132" spans="1:12" ht="15">
+      <c r="A132" s="5"/>
       <c r="B132" s="1" t="s">
         <v>9</v>
       </c>
@@ -4310,11 +4441,12 @@
       <c r="I132" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J132" s="4"/>
+      <c r="J132" s="5"/>
       <c r="K132" s="5"/>
       <c r="L132" s="5"/>
     </row>
-    <row r="133" spans="2:12" ht="15">
+    <row r="133" spans="1:12" ht="15">
+      <c r="A133" s="3"/>
       <c r="B133" s="6" t="s">
         <v>9</v>
       </c>
@@ -4333,11 +4465,12 @@
       <c r="I133" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J133" s="4"/>
+      <c r="J133" s="3"/>
       <c r="K133" s="3"/>
       <c r="L133" s="3"/>
     </row>
-    <row r="134" spans="2:12" ht="15">
+    <row r="134" spans="1:12" ht="15">
+      <c r="A134" s="5"/>
       <c r="B134" s="1" t="s">
         <v>9</v>
       </c>
@@ -4356,11 +4489,12 @@
       <c r="I134" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J134" s="4"/>
+      <c r="J134" s="5"/>
       <c r="K134" s="5"/>
       <c r="L134" s="3"/>
     </row>
-    <row r="135" spans="2:12" ht="15">
+    <row r="135" spans="1:12" ht="15">
+      <c r="A135" s="3"/>
       <c r="B135" s="6" t="s">
         <v>3</v>
       </c>
@@ -4379,11 +4513,12 @@
       <c r="I135" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J135" s="4"/>
+      <c r="J135" s="3"/>
       <c r="K135" s="3"/>
       <c r="L135" s="5"/>
     </row>
-    <row r="136" spans="2:12" ht="15">
+    <row r="136" spans="1:12" ht="15">
+      <c r="A136" s="5"/>
       <c r="B136" s="1" t="s">
         <v>9</v>
       </c>
@@ -4402,11 +4537,12 @@
       <c r="I136" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J136" s="4"/>
+      <c r="J136" s="5"/>
       <c r="K136" s="5"/>
       <c r="L136" s="3"/>
     </row>
-    <row r="137" spans="2:12" ht="15">
+    <row r="137" spans="1:12" ht="15">
+      <c r="A137" s="5"/>
       <c r="B137" s="6" t="s">
         <v>9</v>
       </c>
@@ -4425,11 +4561,12 @@
       <c r="I137" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J137" s="4"/>
+      <c r="J137" s="5"/>
       <c r="K137" s="5"/>
       <c r="L137" s="3"/>
     </row>
-    <row r="138" spans="2:12" ht="15">
+    <row r="138" spans="1:12" ht="15">
+      <c r="A138" s="5"/>
       <c r="B138" s="1" t="s">
         <v>9</v>
       </c>
@@ -4448,11 +4585,12 @@
       <c r="I138" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J138" s="4"/>
+      <c r="J138" s="5"/>
       <c r="K138" s="5"/>
       <c r="L138" s="5"/>
     </row>
-    <row r="139" spans="2:12" ht="15">
+    <row r="139" spans="1:12" ht="15">
+      <c r="A139" s="5"/>
       <c r="B139" s="6" t="s">
         <v>9</v>
       </c>
@@ -4471,11 +4609,12 @@
       <c r="I139" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J139" s="4"/>
+      <c r="J139" s="5"/>
       <c r="K139" s="5"/>
       <c r="L139" s="3"/>
     </row>
-    <row r="140" spans="2:12" ht="15">
+    <row r="140" spans="1:12" ht="15">
+      <c r="A140" s="5"/>
       <c r="B140" s="1" t="s">
         <v>9</v>
       </c>
@@ -4494,11 +4633,12 @@
       <c r="I140" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J140" s="4"/>
+      <c r="J140" s="5"/>
       <c r="K140" s="5"/>
       <c r="L140" s="3"/>
     </row>
-    <row r="141" spans="2:12" ht="15">
+    <row r="141" spans="1:12" ht="15">
+      <c r="A141" s="5"/>
       <c r="B141" s="6" t="s">
         <v>9</v>
       </c>
@@ -4517,11 +4657,12 @@
       <c r="I141" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J141" s="4"/>
+      <c r="J141" s="5"/>
       <c r="K141" s="5"/>
       <c r="L141" s="5"/>
     </row>
-    <row r="142" spans="2:12" ht="15">
+    <row r="142" spans="1:12" ht="15">
+      <c r="A142" s="5"/>
       <c r="B142" s="1" t="s">
         <v>3</v>
       </c>
@@ -4540,11 +4681,12 @@
       <c r="I142" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J142" s="4"/>
+      <c r="J142" s="5"/>
       <c r="K142" s="5"/>
       <c r="L142" s="3"/>
     </row>
-    <row r="143" spans="2:12" ht="15">
+    <row r="143" spans="1:12" ht="15">
+      <c r="A143" s="5"/>
       <c r="B143" s="6" t="s">
         <v>9</v>
       </c>
@@ -4563,11 +4705,12 @@
       <c r="I143" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J143" s="4"/>
+      <c r="J143" s="5"/>
       <c r="K143" s="5"/>
       <c r="L143" s="3"/>
     </row>
-    <row r="144" spans="2:12" ht="15">
+    <row r="144" spans="1:12" ht="15">
+      <c r="A144" s="5"/>
       <c r="B144" s="1" t="s">
         <v>9</v>
       </c>
@@ -4586,11 +4729,12 @@
       <c r="I144" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J144" s="4"/>
+      <c r="J144" s="5"/>
       <c r="K144" s="5"/>
       <c r="L144" s="5"/>
     </row>
-    <row r="145" spans="2:12" ht="15">
+    <row r="145" spans="1:12" ht="15">
+      <c r="A145" s="5"/>
       <c r="B145" s="6" t="s">
         <v>9</v>
       </c>
@@ -4609,11 +4753,12 @@
       <c r="I145" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J145" s="4"/>
+      <c r="J145" s="5"/>
       <c r="K145" s="5"/>
       <c r="L145" s="3"/>
     </row>
-    <row r="146" spans="2:12" ht="15">
+    <row r="146" spans="1:12" ht="15">
+      <c r="A146" s="5"/>
       <c r="B146" s="1" t="s">
         <v>3</v>
       </c>
@@ -4632,11 +4777,12 @@
       <c r="I146" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J146" s="4"/>
+      <c r="J146" s="5"/>
       <c r="K146" s="5"/>
       <c r="L146" s="3"/>
     </row>
-    <row r="147" spans="2:12" ht="15">
+    <row r="147" spans="1:12" ht="15">
+      <c r="A147" s="3"/>
       <c r="B147" s="6" t="s">
         <v>3</v>
       </c>
@@ -4655,11 +4801,12 @@
       <c r="I147" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J147" s="4"/>
+      <c r="J147" s="3"/>
       <c r="K147" s="3"/>
       <c r="L147" s="5"/>
     </row>
-    <row r="148" spans="2:12" ht="15">
+    <row r="148" spans="1:12" ht="15">
+      <c r="A148" s="3"/>
       <c r="B148" s="1" t="s">
         <v>9</v>
       </c>
@@ -4678,11 +4825,12 @@
       <c r="I148" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J148" s="4"/>
+      <c r="J148" s="3"/>
       <c r="K148" s="3"/>
       <c r="L148" s="3"/>
     </row>
-    <row r="149" spans="2:12" ht="15">
+    <row r="149" spans="1:12" ht="15">
+      <c r="A149" s="3"/>
       <c r="B149" s="6" t="s">
         <v>3</v>
       </c>
@@ -4701,11 +4849,12 @@
       <c r="I149" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J149" s="4"/>
+      <c r="J149" s="3"/>
       <c r="K149" s="3"/>
       <c r="L149" s="3"/>
     </row>
-    <row r="150" spans="2:12" ht="15">
+    <row r="150" spans="1:12" ht="15">
+      <c r="A150" s="5"/>
       <c r="B150" s="1" t="s">
         <v>9</v>
       </c>
@@ -4724,11 +4873,12 @@
       <c r="I150" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J150" s="4"/>
+      <c r="J150" s="5"/>
       <c r="K150" s="5"/>
       <c r="L150" s="5"/>
     </row>
-    <row r="151" spans="2:12" ht="15">
+    <row r="151" spans="1:12" ht="15">
+      <c r="A151" s="3"/>
       <c r="B151" s="6" t="s">
         <v>3</v>
       </c>
@@ -4747,11 +4897,12 @@
       <c r="I151" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J151" s="4"/>
+      <c r="J151" s="3"/>
       <c r="K151" s="3"/>
       <c r="L151" s="3"/>
     </row>
-    <row r="152" spans="2:12" ht="15">
+    <row r="152" spans="1:12" ht="15">
+      <c r="A152" s="5"/>
       <c r="B152" s="1" t="s">
         <v>9</v>
       </c>
@@ -4770,11 +4921,12 @@
       <c r="I152" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J152" s="4"/>
+      <c r="J152" s="5"/>
       <c r="K152" s="5"/>
       <c r="L152" s="3"/>
     </row>
-    <row r="153" spans="2:12" ht="15">
+    <row r="153" spans="1:12" ht="15">
+      <c r="A153" s="3"/>
       <c r="B153" s="6" t="s">
         <v>9</v>
       </c>
@@ -4793,11 +4945,12 @@
       <c r="I153" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J153" s="4"/>
+      <c r="J153" s="3"/>
       <c r="K153" s="3"/>
       <c r="L153" s="5"/>
     </row>
-    <row r="154" spans="2:12" ht="15">
+    <row r="154" spans="1:12" ht="15">
+      <c r="A154" s="5"/>
       <c r="B154" s="1" t="s">
         <v>3</v>
       </c>
@@ -4816,11 +4969,12 @@
       <c r="I154" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J154" s="4"/>
+      <c r="J154" s="5"/>
       <c r="K154" s="5"/>
       <c r="L154" s="3"/>
     </row>
-    <row r="155" spans="2:12" ht="15">
+    <row r="155" spans="1:12" ht="15">
+      <c r="A155" s="3"/>
       <c r="B155" s="6" t="s">
         <v>3</v>
       </c>
@@ -4839,11 +4993,12 @@
       <c r="I155" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J155" s="4"/>
+      <c r="J155" s="3"/>
       <c r="K155" s="3"/>
       <c r="L155" s="3"/>
     </row>
-    <row r="156" spans="2:12" ht="15">
+    <row r="156" spans="1:12" ht="15">
+      <c r="A156" s="5"/>
       <c r="B156" s="1" t="s">
         <v>3</v>
       </c>
@@ -4862,11 +5017,12 @@
       <c r="I156" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J156" s="4"/>
+      <c r="J156" s="5"/>
       <c r="K156" s="5"/>
       <c r="L156" s="5"/>
     </row>
-    <row r="157" spans="2:12" ht="15">
+    <row r="157" spans="1:12" ht="15">
+      <c r="A157" s="3"/>
       <c r="B157" s="6" t="s">
         <v>9</v>
       </c>
@@ -4885,11 +5041,12 @@
       <c r="I157" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J157" s="4"/>
+      <c r="J157" s="3"/>
       <c r="K157" s="3"/>
       <c r="L157" s="3"/>
     </row>
-    <row r="158" spans="2:12" ht="15">
+    <row r="158" spans="1:12" ht="15">
+      <c r="A158" s="5"/>
       <c r="B158" s="1" t="s">
         <v>3</v>
       </c>
@@ -4908,11 +5065,11 @@
       <c r="I158" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J158" s="4"/>
+      <c r="J158" s="5"/>
       <c r="K158" s="5"/>
       <c r="L158" s="3"/>
     </row>
-    <row r="159" spans="2:12" ht="15">
+    <row r="159" spans="1:12" ht="15">
       <c r="B159" s="6" t="s">
         <v>3</v>
       </c>
@@ -4931,10 +5088,10 @@
       <c r="I159" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J159" s="4"/>
       <c r="L159" s="5"/>
     </row>
-    <row r="160" spans="2:12" ht="15">
+    <row r="160" spans="1:12" ht="15">
+      <c r="A160" s="5"/>
       <c r="B160" s="1" t="s">
         <v>9</v>
       </c>
@@ -4953,11 +5110,12 @@
       <c r="I160" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J160" s="4"/>
+      <c r="J160" s="5"/>
       <c r="K160" s="5"/>
       <c r="L160" s="3"/>
     </row>
-    <row r="161" spans="2:12" ht="15">
+    <row r="161" spans="1:12" ht="15">
+      <c r="A161" s="3"/>
       <c r="B161" s="6" t="s">
         <v>3</v>
       </c>
@@ -4976,11 +5134,12 @@
       <c r="I161" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J161" s="4"/>
+      <c r="J161" s="3"/>
       <c r="K161" s="3"/>
       <c r="L161" s="3"/>
     </row>
-    <row r="162" spans="2:12" ht="15">
+    <row r="162" spans="1:12" ht="15">
+      <c r="A162" s="5"/>
       <c r="B162" s="1" t="s">
         <v>9</v>
       </c>
@@ -4999,11 +5158,12 @@
       <c r="I162" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J162" s="4"/>
+      <c r="J162" s="5"/>
       <c r="K162" s="5"/>
       <c r="L162" s="5"/>
     </row>
-    <row r="163" spans="2:12" ht="15">
+    <row r="163" spans="1:12" ht="15">
+      <c r="A163" s="3"/>
       <c r="B163" s="6" t="s">
         <v>3</v>
       </c>
@@ -5022,11 +5182,12 @@
       <c r="I163" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J163" s="4"/>
+      <c r="J163" s="3"/>
       <c r="K163" s="3"/>
       <c r="L163" s="3"/>
     </row>
-    <row r="164" spans="2:12" ht="15">
+    <row r="164" spans="1:12" ht="15">
+      <c r="A164" s="5"/>
       <c r="B164" s="1" t="s">
         <v>9</v>
       </c>
@@ -5045,11 +5206,12 @@
       <c r="I164" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J164" s="4"/>
+      <c r="J164" s="5"/>
       <c r="K164" s="5"/>
       <c r="L164" s="3"/>
     </row>
-    <row r="165" spans="2:12" ht="15">
+    <row r="165" spans="1:12" ht="15">
+      <c r="A165" s="3"/>
       <c r="B165" s="6" t="s">
         <v>9</v>
       </c>
@@ -5068,11 +5230,12 @@
       <c r="I165" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J165" s="4"/>
+      <c r="J165" s="3"/>
       <c r="K165" s="3"/>
       <c r="L165" s="5"/>
     </row>
-    <row r="166" spans="2:12" ht="15">
+    <row r="166" spans="1:12" ht="15">
+      <c r="A166" s="5"/>
       <c r="B166" s="1" t="s">
         <v>39</v>
       </c>
@@ -5091,11 +5254,12 @@
       <c r="I166" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J166" s="4"/>
+      <c r="J166" s="5"/>
       <c r="K166" s="5"/>
       <c r="L166" s="3"/>
     </row>
-    <row r="167" spans="2:12" ht="15">
+    <row r="167" spans="1:12" ht="15">
+      <c r="A167" s="5"/>
       <c r="B167" s="6" t="s">
         <v>39</v>
       </c>
@@ -5114,11 +5278,12 @@
       <c r="I167" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J167" s="4"/>
+      <c r="J167" s="5"/>
       <c r="K167" s="5"/>
       <c r="L167" s="3"/>
     </row>
-    <row r="168" spans="2:12" ht="15">
+    <row r="168" spans="1:12" ht="15">
+      <c r="A168" s="3"/>
       <c r="B168" s="1" t="s">
         <v>9</v>
       </c>
@@ -5137,11 +5302,12 @@
       <c r="I168" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J168" s="4"/>
+      <c r="J168" s="3"/>
       <c r="K168" s="3"/>
       <c r="L168" s="5"/>
     </row>
-    <row r="169" spans="2:12" ht="15">
+    <row r="169" spans="1:12" ht="15">
+      <c r="A169" s="5"/>
       <c r="B169" s="6" t="s">
         <v>3</v>
       </c>
@@ -5160,11 +5326,12 @@
       <c r="I169" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J169" s="4"/>
+      <c r="J169" s="5"/>
       <c r="K169" s="5"/>
       <c r="L169" s="3"/>
     </row>
-    <row r="170" spans="2:12" ht="15">
+    <row r="170" spans="1:12" ht="15">
+      <c r="A170" s="3"/>
       <c r="B170" s="1" t="s">
         <v>3</v>
       </c>
@@ -5183,11 +5350,12 @@
       <c r="I170" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J170" s="4"/>
+      <c r="J170" s="3"/>
       <c r="K170" s="3"/>
       <c r="L170" s="3"/>
     </row>
-    <row r="171" spans="2:12" ht="30">
+    <row r="171" spans="1:12" ht="30">
+      <c r="A171" s="5"/>
       <c r="B171" s="6" t="s">
         <v>3</v>
       </c>
@@ -5206,11 +5374,12 @@
       <c r="I171" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J171" s="4"/>
+      <c r="J171" s="5"/>
       <c r="K171" s="5"/>
       <c r="L171" s="5"/>
     </row>
-    <row r="172" spans="2:12" ht="15">
+    <row r="172" spans="1:12" ht="15">
+      <c r="A172" s="3"/>
       <c r="B172" s="1" t="s">
         <v>3</v>
       </c>
@@ -5229,11 +5398,12 @@
       <c r="I172" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J172" s="4"/>
+      <c r="J172" s="3"/>
       <c r="K172" s="3"/>
       <c r="L172" s="3"/>
     </row>
-    <row r="173" spans="2:12" ht="30">
+    <row r="173" spans="1:12" ht="30">
+      <c r="A173" s="5"/>
       <c r="B173" s="6" t="s">
         <v>3</v>
       </c>
@@ -5252,11 +5422,12 @@
       <c r="I173" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J173" s="4"/>
+      <c r="J173" s="5"/>
       <c r="K173" s="5"/>
       <c r="L173" s="3"/>
     </row>
-    <row r="174" spans="2:12" ht="15">
+    <row r="174" spans="1:12" ht="15">
+      <c r="A174" s="3"/>
       <c r="B174" s="1" t="s">
         <v>9</v>
       </c>
@@ -5275,11 +5446,12 @@
       <c r="I174" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J174" s="4"/>
+      <c r="J174" s="3"/>
       <c r="K174" s="3"/>
       <c r="L174" s="5"/>
     </row>
-    <row r="175" spans="2:12" ht="15">
+    <row r="175" spans="1:12" ht="15">
+      <c r="A175" s="5"/>
       <c r="B175" s="6" t="s">
         <v>39</v>
       </c>
@@ -5298,11 +5470,12 @@
       <c r="I175" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J175" s="4"/>
+      <c r="J175" s="5"/>
       <c r="K175" s="5"/>
       <c r="L175" s="3"/>
     </row>
-    <row r="176" spans="2:12" ht="30">
+    <row r="176" spans="1:12" ht="30">
+      <c r="A176" s="3"/>
       <c r="B176" s="1" t="s">
         <v>39</v>
       </c>
@@ -5321,11 +5494,12 @@
       <c r="I176" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J176" s="4"/>
+      <c r="J176" s="3"/>
       <c r="K176" s="3"/>
       <c r="L176" s="3"/>
     </row>
-    <row r="177" spans="2:12" ht="15">
+    <row r="177" spans="1:12" ht="15">
+      <c r="A177" s="5"/>
       <c r="B177" s="6" t="s">
         <v>39</v>
       </c>
@@ -5344,11 +5518,12 @@
       <c r="I177" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J177" s="4"/>
+      <c r="J177" s="5"/>
       <c r="K177" s="5"/>
       <c r="L177" s="5"/>
     </row>
-    <row r="178" spans="2:12" ht="15">
+    <row r="178" spans="1:12" ht="15">
+      <c r="A178" s="5"/>
       <c r="B178" s="1" t="s">
         <v>39</v>
       </c>
@@ -5367,11 +5542,12 @@
       <c r="I178" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J178" s="4"/>
+      <c r="J178" s="5"/>
       <c r="K178" s="5"/>
       <c r="L178" s="3"/>
     </row>
-    <row r="179" spans="2:12" ht="15">
+    <row r="179" spans="1:12" ht="15">
+      <c r="A179" s="5"/>
       <c r="B179" s="6" t="s">
         <v>39</v>
       </c>
@@ -5390,11 +5566,12 @@
       <c r="I179" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J179" s="4"/>
+      <c r="J179" s="5"/>
       <c r="K179" s="5"/>
       <c r="L179" s="3"/>
     </row>
-    <row r="180" spans="2:12" ht="15">
+    <row r="180" spans="1:12" ht="15">
+      <c r="A180" s="5"/>
       <c r="B180" s="1" t="s">
         <v>39</v>
       </c>
@@ -5413,11 +5590,12 @@
       <c r="I180" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J180" s="4"/>
+      <c r="J180" s="5"/>
       <c r="K180" s="5"/>
       <c r="L180" s="5"/>
     </row>
-    <row r="181" spans="2:12" ht="30">
+    <row r="181" spans="1:12" ht="30">
+      <c r="A181" s="5"/>
       <c r="B181" s="6" t="s">
         <v>9</v>
       </c>
@@ -5436,11 +5614,12 @@
       <c r="I181" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J181" s="4"/>
+      <c r="J181" s="5"/>
       <c r="K181" s="5"/>
       <c r="L181" s="3"/>
     </row>
-    <row r="182" spans="2:12" ht="15">
+    <row r="182" spans="1:12" ht="15">
+      <c r="A182" s="5"/>
       <c r="B182" s="1" t="s">
         <v>9</v>
       </c>
@@ -5459,11 +5638,12 @@
       <c r="I182" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J182" s="4"/>
+      <c r="J182" s="5"/>
       <c r="K182" s="5"/>
       <c r="L182" s="3"/>
     </row>
-    <row r="183" spans="2:12" ht="30">
+    <row r="183" spans="1:12" ht="30">
+      <c r="A183" s="5"/>
       <c r="B183" s="6" t="s">
         <v>9</v>
       </c>
@@ -5482,11 +5662,12 @@
       <c r="I183" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J183" s="4"/>
+      <c r="J183" s="5"/>
       <c r="K183" s="5"/>
       <c r="L183" s="5"/>
     </row>
-    <row r="184" spans="2:12" ht="15">
+    <row r="184" spans="1:12" ht="15">
+      <c r="A184" s="3"/>
       <c r="B184" s="1" t="s">
         <v>9</v>
       </c>
@@ -5505,11 +5686,12 @@
       <c r="I184" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J184" s="4"/>
+      <c r="J184" s="3"/>
       <c r="K184" s="3"/>
       <c r="L184" s="3"/>
     </row>
-    <row r="185" spans="2:12" ht="15">
+    <row r="185" spans="1:12" ht="15">
+      <c r="A185" s="5"/>
       <c r="B185" s="6" t="s">
         <v>9</v>
       </c>
@@ -5528,11 +5710,12 @@
       <c r="I185" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J185" s="4"/>
+      <c r="J185" s="5"/>
       <c r="K185" s="5"/>
       <c r="L185" s="3"/>
     </row>
-    <row r="186" spans="2:12" ht="30">
+    <row r="186" spans="1:12" ht="30">
+      <c r="A186" s="3"/>
       <c r="B186" s="1" t="s">
         <v>9</v>
       </c>
@@ -5551,11 +5734,12 @@
       <c r="I186" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J186" s="4"/>
+      <c r="J186" s="3"/>
       <c r="K186" s="3"/>
       <c r="L186" s="5"/>
     </row>
-    <row r="187" spans="2:12" ht="30">
+    <row r="187" spans="1:12" ht="30">
+      <c r="A187" s="5"/>
       <c r="B187" s="6" t="s">
         <v>3</v>
       </c>
@@ -5574,11 +5758,12 @@
       <c r="I187" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J187" s="4"/>
+      <c r="J187" s="5"/>
       <c r="K187" s="5"/>
       <c r="L187" s="3"/>
     </row>
-    <row r="188" spans="2:12" ht="15">
+    <row r="188" spans="1:12" ht="15">
+      <c r="A188" s="5"/>
       <c r="B188" s="1" t="s">
         <v>3</v>
       </c>
@@ -5597,11 +5782,12 @@
       <c r="I188" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J188" s="4"/>
+      <c r="J188" s="5"/>
       <c r="K188" s="5"/>
       <c r="L188" s="3"/>
     </row>
-    <row r="189" spans="2:12" ht="15">
+    <row r="189" spans="1:12" ht="15">
+      <c r="A189" s="5"/>
       <c r="B189" s="6" t="s">
         <v>3</v>
       </c>
@@ -5620,11 +5806,12 @@
       <c r="I189" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J189" s="4"/>
+      <c r="J189" s="5"/>
       <c r="K189" s="5"/>
       <c r="L189" s="5"/>
     </row>
-    <row r="190" spans="2:12" ht="15">
+    <row r="190" spans="1:12" ht="15">
+      <c r="A190" s="5"/>
       <c r="B190" s="1" t="s">
         <v>3</v>
       </c>
@@ -5643,11 +5830,12 @@
       <c r="I190" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J190" s="4"/>
+      <c r="J190" s="5"/>
       <c r="K190" s="5"/>
       <c r="L190" s="3"/>
     </row>
-    <row r="191" spans="2:12" ht="15">
+    <row r="191" spans="1:12" ht="15">
+      <c r="A191" s="5"/>
       <c r="B191" s="6" t="s">
         <v>3</v>
       </c>
@@ -5666,11 +5854,12 @@
       <c r="I191" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J191" s="4"/>
+      <c r="J191" s="5"/>
       <c r="K191" s="5"/>
       <c r="L191" s="3"/>
     </row>
-    <row r="192" spans="2:12" ht="15">
+    <row r="192" spans="1:12" ht="15">
+      <c r="A192" s="5"/>
       <c r="B192" s="1" t="s">
         <v>3</v>
       </c>
@@ -5689,11 +5878,12 @@
       <c r="I192" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J192" s="4"/>
+      <c r="J192" s="5"/>
       <c r="K192" s="5"/>
       <c r="L192" s="5"/>
     </row>
-    <row r="193" spans="2:12" ht="15">
+    <row r="193" spans="1:12" ht="15">
+      <c r="A193" s="5"/>
       <c r="B193" s="6" t="s">
         <v>9</v>
       </c>
@@ -5712,11 +5902,12 @@
       <c r="I193" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J193" s="4"/>
+      <c r="J193" s="5"/>
       <c r="K193" s="5"/>
       <c r="L193" s="3"/>
     </row>
-    <row r="194" spans="2:12" ht="15">
+    <row r="194" spans="1:12" ht="15">
+      <c r="A194" s="3"/>
       <c r="B194" s="1" t="s">
         <v>9</v>
       </c>
@@ -5735,11 +5926,12 @@
       <c r="I194" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J194" s="4"/>
+      <c r="J194" s="3"/>
       <c r="K194" s="3"/>
       <c r="L194" s="3"/>
     </row>
-    <row r="195" spans="2:12" ht="15">
+    <row r="195" spans="1:12" ht="15">
+      <c r="A195" s="5"/>
       <c r="B195" s="6" t="s">
         <v>9</v>
       </c>
@@ -5758,11 +5950,12 @@
       <c r="I195" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J195" s="4"/>
+      <c r="J195" s="5"/>
       <c r="K195" s="5"/>
       <c r="L195" s="5"/>
     </row>
-    <row r="196" spans="2:12" ht="15">
+    <row r="196" spans="1:12" ht="15">
+      <c r="A196" s="3"/>
       <c r="B196" s="1" t="s">
         <v>9</v>
       </c>
@@ -5781,11 +5974,12 @@
       <c r="I196" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J196" s="4"/>
+      <c r="J196" s="3"/>
       <c r="K196" s="3"/>
       <c r="L196" s="3"/>
     </row>
-    <row r="197" spans="2:12" ht="15">
+    <row r="197" spans="1:12" ht="15">
+      <c r="A197" s="5"/>
       <c r="B197" s="6" t="s">
         <v>9</v>
       </c>
@@ -5804,11 +5998,12 @@
       <c r="I197" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J197" s="4"/>
+      <c r="J197" s="5"/>
       <c r="K197" s="5"/>
       <c r="L197" s="3"/>
     </row>
-    <row r="198" spans="2:12" ht="15">
+    <row r="198" spans="1:12" ht="15">
+      <c r="A198" s="3"/>
       <c r="B198" s="1" t="s">
         <v>9</v>
       </c>
@@ -5827,11 +6022,12 @@
       <c r="I198" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J198" s="4"/>
+      <c r="J198" s="3"/>
       <c r="K198" s="3"/>
       <c r="L198" s="5"/>
     </row>
-    <row r="199" spans="2:12" ht="15">
+    <row r="199" spans="1:12" ht="15">
+      <c r="A199" s="5"/>
       <c r="B199" s="6" t="s">
         <v>9</v>
       </c>
@@ -5850,11 +6046,12 @@
       <c r="I199" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J199" s="4"/>
+      <c r="J199" s="5"/>
       <c r="K199" s="5"/>
       <c r="L199" s="3"/>
     </row>
-    <row r="200" spans="2:12" ht="15">
+    <row r="200" spans="1:12" ht="15">
+      <c r="A200" s="3"/>
       <c r="B200" s="1" t="s">
         <v>3</v>
       </c>
@@ -5873,11 +6070,12 @@
       <c r="I200" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J200" s="4"/>
+      <c r="J200" s="3"/>
       <c r="K200" s="3"/>
       <c r="L200" s="3"/>
     </row>
-    <row r="201" spans="2:12" ht="15">
+    <row r="201" spans="1:12" ht="15">
+      <c r="A201" s="5"/>
       <c r="B201" s="6" t="s">
         <v>9</v>
       </c>
@@ -5896,11 +6094,12 @@
       <c r="I201" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J201" s="4"/>
+      <c r="J201" s="5"/>
       <c r="K201" s="5"/>
       <c r="L201" s="5"/>
     </row>
-    <row r="202" spans="2:12" ht="60">
+    <row r="202" spans="1:12" ht="60">
+      <c r="A202" s="3"/>
       <c r="B202" s="1" t="s">
         <v>9</v>
       </c>
@@ -5919,11 +6118,12 @@
       <c r="I202" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J202" s="4"/>
+      <c r="J202" s="3"/>
       <c r="K202" s="3"/>
       <c r="L202" s="3"/>
     </row>
-    <row r="203" spans="2:12" ht="60">
+    <row r="203" spans="1:12" ht="60">
+      <c r="A203" s="5"/>
       <c r="B203" s="6" t="s">
         <v>9</v>
       </c>
@@ -5942,11 +6142,12 @@
       <c r="I203" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J203" s="4"/>
+      <c r="J203" s="5"/>
       <c r="K203" s="5"/>
       <c r="L203" s="3"/>
     </row>
-    <row r="204" spans="2:12" ht="15">
+    <row r="204" spans="1:12" ht="15">
+      <c r="A204" s="3"/>
       <c r="B204" s="1" t="s">
         <v>9</v>
       </c>
@@ -5965,11 +6166,12 @@
       <c r="I204" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J204" s="4"/>
+      <c r="J204" s="3"/>
       <c r="K204" s="3"/>
       <c r="L204" s="5"/>
     </row>
-    <row r="205" spans="2:12" ht="15">
+    <row r="205" spans="1:12" ht="15">
+      <c r="A205" s="5"/>
       <c r="B205" s="6" t="s">
         <v>9</v>
       </c>
@@ -5988,11 +6190,12 @@
       <c r="I205" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J205" s="4"/>
+      <c r="J205" s="5"/>
       <c r="K205" s="5"/>
       <c r="L205" s="3"/>
     </row>
-    <row r="206" spans="2:12" ht="15">
+    <row r="206" spans="1:12" ht="15">
+      <c r="A206" s="3"/>
       <c r="B206" s="1" t="s">
         <v>9</v>
       </c>
@@ -6011,11 +6214,12 @@
       <c r="I206" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J206" s="4"/>
+      <c r="J206" s="3"/>
       <c r="K206" s="3"/>
       <c r="L206" s="3"/>
     </row>
-    <row r="207" spans="2:12" ht="15">
+    <row r="207" spans="1:12" ht="15">
+      <c r="A207" s="5"/>
       <c r="B207" s="6" t="s">
         <v>9</v>
       </c>
@@ -6034,11 +6238,12 @@
       <c r="I207" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J207" s="4"/>
+      <c r="J207" s="5"/>
       <c r="K207" s="5"/>
       <c r="L207" s="5"/>
     </row>
-    <row r="208" spans="2:12" ht="30">
+    <row r="208" spans="1:12" ht="30">
+      <c r="A208" s="5"/>
       <c r="B208" s="1" t="s">
         <v>9</v>
       </c>
@@ -6057,11 +6262,12 @@
       <c r="I208" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J208" s="4"/>
+      <c r="J208" s="5"/>
       <c r="K208" s="5"/>
       <c r="L208" s="3"/>
     </row>
-    <row r="209" spans="2:12" ht="30">
+    <row r="209" spans="1:12" ht="30">
+      <c r="A209" s="5"/>
       <c r="B209" s="6" t="s">
         <v>3</v>
       </c>
@@ -6080,11 +6286,12 @@
       <c r="I209" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J209" s="4"/>
+      <c r="J209" s="5"/>
       <c r="K209" s="5"/>
       <c r="L209" s="3"/>
     </row>
-    <row r="210" spans="2:12" ht="30">
+    <row r="210" spans="1:12" ht="30">
+      <c r="A210" s="3"/>
       <c r="B210" s="1" t="s">
         <v>39</v>
       </c>
@@ -6103,11 +6310,12 @@
       <c r="I210" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J210" s="4"/>
+      <c r="J210" s="3"/>
       <c r="K210" s="3"/>
       <c r="L210" s="5"/>
     </row>
-    <row r="211" spans="2:12" ht="15">
+    <row r="211" spans="1:12" ht="15">
+      <c r="A211" s="5"/>
       <c r="B211" s="6" t="s">
         <v>9</v>
       </c>
@@ -6126,11 +6334,12 @@
       <c r="I211" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J211" s="4"/>
+      <c r="J211" s="5"/>
       <c r="K211" s="5"/>
       <c r="L211" s="3"/>
     </row>
-    <row r="212" spans="2:12" ht="30">
+    <row r="212" spans="1:12" ht="30">
+      <c r="A212" s="5"/>
       <c r="B212" s="1" t="s">
         <v>9</v>
       </c>
@@ -6149,11 +6358,12 @@
       <c r="I212" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J212" s="4"/>
+      <c r="J212" s="5"/>
       <c r="K212" s="5"/>
       <c r="L212" s="3"/>
     </row>
-    <row r="213" spans="2:12" ht="30">
+    <row r="213" spans="1:12" ht="30">
+      <c r="A213" s="5"/>
       <c r="B213" s="6" t="s">
         <v>39</v>
       </c>
@@ -6172,11 +6382,12 @@
       <c r="I213" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J213" s="4"/>
+      <c r="J213" s="5"/>
       <c r="K213" s="5"/>
       <c r="L213" s="5"/>
     </row>
-    <row r="214" spans="2:12" ht="15">
+    <row r="214" spans="1:12" ht="15">
+      <c r="A214" s="5"/>
       <c r="B214" s="1" t="s">
         <v>39</v>
       </c>
@@ -6195,11 +6406,12 @@
       <c r="I214" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J214" s="4"/>
+      <c r="J214" s="5"/>
       <c r="K214" s="5"/>
       <c r="L214" s="3"/>
     </row>
-    <row r="215" spans="2:12" ht="15">
+    <row r="215" spans="1:12" ht="15">
+      <c r="A215" s="5"/>
       <c r="B215" s="6" t="s">
         <v>39</v>
       </c>
@@ -6218,11 +6430,12 @@
       <c r="I215" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J215" s="4"/>
+      <c r="J215" s="5"/>
       <c r="K215" s="5"/>
       <c r="L215" s="3"/>
     </row>
-    <row r="216" spans="2:12" ht="15">
+    <row r="216" spans="1:12" ht="15">
+      <c r="A216" s="5"/>
       <c r="B216" s="1" t="s">
         <v>39</v>
       </c>
@@ -6241,11 +6454,12 @@
       <c r="I216" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J216" s="4"/>
+      <c r="J216" s="5"/>
       <c r="K216" s="5"/>
       <c r="L216" s="5"/>
     </row>
-    <row r="217" spans="2:12" ht="15">
+    <row r="217" spans="1:12" ht="15">
+      <c r="A217" s="5"/>
       <c r="B217" s="6" t="s">
         <v>39</v>
       </c>
@@ -6264,11 +6478,12 @@
       <c r="I217" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J217" s="4"/>
+      <c r="J217" s="5"/>
       <c r="K217" s="5"/>
       <c r="L217" s="3"/>
     </row>
-    <row r="218" spans="2:12" ht="15">
+    <row r="218" spans="1:12" ht="15">
+      <c r="A218" s="5"/>
       <c r="B218" s="1" t="s">
         <v>39</v>
       </c>
@@ -6287,11 +6502,12 @@
       <c r="I218" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J218" s="4"/>
+      <c r="J218" s="5"/>
       <c r="K218" s="5"/>
       <c r="L218" s="3"/>
     </row>
-    <row r="219" spans="2:12" ht="15">
+    <row r="219" spans="1:12" ht="15">
+      <c r="A219" s="5"/>
       <c r="B219" s="6" t="s">
         <v>39</v>
       </c>
@@ -6310,11 +6526,12 @@
       <c r="I219" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J219" s="4"/>
+      <c r="J219" s="5"/>
       <c r="K219" s="5"/>
       <c r="L219" s="5"/>
     </row>
-    <row r="220" spans="2:12" ht="30">
+    <row r="220" spans="1:12" ht="30">
+      <c r="A220" s="3"/>
       <c r="B220" s="1" t="s">
         <v>3</v>
       </c>
@@ -6333,11 +6550,12 @@
       <c r="I220" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J220" s="4"/>
+      <c r="J220" s="3"/>
       <c r="K220" s="3"/>
       <c r="L220" s="3"/>
     </row>
-    <row r="221" spans="2:12" ht="15">
+    <row r="221" spans="1:12" ht="15">
+      <c r="A221" s="5"/>
       <c r="B221" s="6" t="s">
         <v>39</v>
       </c>
@@ -6356,11 +6574,12 @@
       <c r="I221" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J221" s="4"/>
+      <c r="J221" s="5"/>
       <c r="K221" s="5"/>
       <c r="L221" s="3"/>
     </row>
-    <row r="222" spans="2:12" ht="30">
+    <row r="222" spans="1:12" ht="30">
+      <c r="A222" s="3"/>
       <c r="B222" s="1" t="s">
         <v>9</v>
       </c>
@@ -6379,11 +6598,12 @@
       <c r="I222" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J222" s="4"/>
+      <c r="J222" s="3"/>
       <c r="K222" s="3"/>
       <c r="L222" s="5"/>
     </row>
-    <row r="223" spans="2:12" ht="15">
+    <row r="223" spans="1:12" ht="15">
+      <c r="A223" s="5"/>
       <c r="B223" s="6" t="s">
         <v>39</v>
       </c>
@@ -6402,11 +6622,12 @@
       <c r="I223" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J223" s="4"/>
+      <c r="J223" s="5"/>
       <c r="K223" s="5"/>
       <c r="L223" s="3"/>
     </row>
-    <row r="224" spans="2:12" ht="15">
+    <row r="224" spans="1:12" ht="15">
+      <c r="A224" s="3"/>
       <c r="B224" s="1" t="s">
         <v>9</v>
       </c>
@@ -6425,11 +6646,12 @@
       <c r="I224" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J224" s="4"/>
+      <c r="J224" s="3"/>
       <c r="K224" s="3"/>
       <c r="L224" s="3"/>
     </row>
-    <row r="225" spans="2:12" ht="15">
+    <row r="225" spans="1:12" ht="15">
+      <c r="A225" s="5"/>
       <c r="B225" s="6" t="s">
         <v>39</v>
       </c>
@@ -6448,11 +6670,12 @@
       <c r="I225" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J225" s="4"/>
+      <c r="J225" s="5"/>
       <c r="K225" s="5"/>
       <c r="L225" s="5"/>
     </row>
-    <row r="226" spans="2:12" ht="15">
+    <row r="226" spans="1:12" ht="15">
+      <c r="A226" s="3"/>
       <c r="B226" s="1" t="s">
         <v>39</v>
       </c>
@@ -6471,11 +6694,12 @@
       <c r="I226" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J226" s="4"/>
+      <c r="J226" s="3"/>
       <c r="K226" s="3"/>
       <c r="L226" s="3"/>
     </row>
-    <row r="227" spans="2:12" ht="15">
+    <row r="227" spans="1:12" ht="15">
+      <c r="A227" s="5"/>
       <c r="B227" s="6" t="s">
         <v>9</v>
       </c>
@@ -6494,11 +6718,12 @@
       <c r="I227" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J227" s="4"/>
+      <c r="J227" s="5"/>
       <c r="K227" s="5"/>
       <c r="L227" s="3"/>
     </row>
-    <row r="228" spans="2:12" ht="15">
+    <row r="228" spans="1:12" ht="15">
+      <c r="A228" s="3"/>
       <c r="B228" s="1" t="s">
         <v>39</v>
       </c>
@@ -6517,11 +6742,12 @@
       <c r="I228" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J228" s="4"/>
+      <c r="J228" s="3"/>
       <c r="K228" s="3"/>
       <c r="L228" s="5"/>
     </row>
-    <row r="229" spans="2:12" ht="15">
+    <row r="229" spans="1:12" ht="15">
+      <c r="A229" s="5"/>
       <c r="B229" s="6" t="s">
         <v>39</v>
       </c>
@@ -6540,11 +6766,12 @@
       <c r="I229" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J229" s="4"/>
+      <c r="J229" s="5"/>
       <c r="K229" s="5"/>
       <c r="L229" s="3"/>
     </row>
-    <row r="230" spans="2:12" ht="15">
+    <row r="230" spans="1:12" ht="15">
+      <c r="A230" s="5"/>
       <c r="B230" s="1" t="s">
         <v>39</v>
       </c>
@@ -6563,11 +6790,12 @@
       <c r="I230" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J230" s="4"/>
+      <c r="J230" s="5"/>
       <c r="K230" s="5"/>
       <c r="L230" s="3"/>
     </row>
-    <row r="231" spans="2:12" ht="15">
+    <row r="231" spans="1:12" ht="15">
+      <c r="A231" s="3"/>
       <c r="B231" s="6" t="s">
         <v>9</v>
       </c>
@@ -6586,11 +6814,12 @@
       <c r="I231" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J231" s="4"/>
+      <c r="J231" s="3"/>
       <c r="K231" s="3"/>
       <c r="L231" s="5"/>
     </row>
-    <row r="232" spans="2:12" ht="15">
+    <row r="232" spans="1:12" ht="15">
+      <c r="A232" s="5"/>
       <c r="B232" s="1" t="s">
         <v>3</v>
       </c>
@@ -6609,11 +6838,12 @@
       <c r="I232" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J232" s="4"/>
+      <c r="J232" s="5"/>
       <c r="K232" s="5"/>
       <c r="L232" s="3"/>
     </row>
-    <row r="233" spans="2:12" ht="15">
+    <row r="233" spans="1:12" ht="15">
+      <c r="A233" s="5"/>
       <c r="B233" s="6" t="s">
         <v>3</v>
       </c>
@@ -6632,11 +6862,12 @@
       <c r="I233" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J233" s="4"/>
+      <c r="J233" s="5"/>
       <c r="K233" s="5"/>
       <c r="L233" s="3"/>
     </row>
-    <row r="234" spans="2:12" ht="30">
+    <row r="234" spans="1:12" ht="30">
+      <c r="A234" s="5"/>
       <c r="B234" s="1" t="s">
         <v>3</v>
       </c>
@@ -6655,15 +6886,15 @@
       <c r="I234" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J234" s="4"/>
+      <c r="J234" s="5"/>
       <c r="K234" s="5"/>
       <c r="L234" s="5"/>
     </row>
-    <row r="235" spans="2:12" ht="14">
+    <row r="235" spans="1:12" ht="14">
       <c r="K235" s="5"/>
       <c r="L235" s="3"/>
     </row>
-    <row r="236" spans="2:12" ht="14">
+    <row r="236" spans="1:12" ht="14">
       <c r="B236" s="1"/>
       <c r="C236" s="7"/>
       <c r="D236" s="7"/>
@@ -6676,10 +6907,10 @@
       <c r="K236" s="5"/>
       <c r="L236" s="3"/>
     </row>
-    <row r="237" spans="2:12" ht="13"/>
-    <row r="238" spans="2:12" ht="13"/>
-    <row r="239" spans="2:12" ht="13"/>
-    <row r="240" spans="2:12" ht="13"/>
+    <row r="237" spans="1:12" ht="13"/>
+    <row r="238" spans="1:12" ht="13"/>
+    <row r="239" spans="1:12" ht="13"/>
+    <row r="240" spans="1:12" ht="13"/>
     <row r="241" spans="8:8" ht="13"/>
     <row r="242" spans="8:8" ht="13"/>
     <row r="243" spans="8:8" ht="13"/>
@@ -9089,7 +9320,7 @@
       <c r="H1048" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J248">
+  <conditionalFormatting sqref="I235:J248 I2:I234">
     <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Funciona">
       <formula>NOT(ISERROR(SEARCH("Funciona",I2)))</formula>
     </cfRule>
@@ -9111,7 +9342,7 @@
       <formula1>"Acceso,Buscador,Control Compras,Control Parental,Navegación,NPVR,Perfiles,Rep. Canal Líneal,Reproducción,TimeShift,Transacción,Claro Música,Trickplay,Social y Settings"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:J234 I236:J236" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I236:J236 I2:I234" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Funciona,Falla nueva,Falla persiste,N/A,Pendiente,Por ejecutar,"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>